<commit_message>
Another edit to template
</commit_message>
<xml_diff>
--- a/report_templates/Cattle-Deaths-Template.xlsx
+++ b/report_templates/Cattle-Deaths-Template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30619"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F3E2F9A2-E688-4FF7-864B-9220AFD20634}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{49961780-C035-4DCE-808B-EA99602BA349}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -137,10 +137,10 @@
     <t>Country</t>
   </si>
   <si>
-    <t>Age at Death in Months</t>
+    <t>County</t>
   </si>
   <si>
-    <t>Premise Type Groups</t>
+    <t>Age at Death in Months</t>
   </si>
   <si>
     <t>Number of Deaths</t>
@@ -510,101 +510,101 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="4" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="4" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="3" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="3" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1920,117 +1920,117 @@
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
-      <c r="E1" s="29" t="s">
+      <c r="E1" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
       <c r="H1" s="3"/>
       <c r="I1" s="3"/>
-      <c r="J1" s="4"/>
+      <c r="J1" s="26"/>
       <c r="K1" s="3"/>
-      <c r="L1" s="5"/>
+      <c r="L1" s="4"/>
     </row>
     <row r="2" spans="1:12" ht="8.1" customHeight="1">
-      <c r="A2" s="6"/>
-      <c r="B2" s="10"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="9"/>
-      <c r="J2" s="10"/>
-      <c r="K2" s="10"/>
-      <c r="L2" s="11"/>
+      <c r="A2" s="5"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="8"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
+      <c r="L2" s="10"/>
     </row>
     <row r="3" spans="1:12" ht="50.25" customHeight="1">
-      <c r="A3" s="12"/>
-      <c r="B3" s="28" t="s">
+      <c r="A3" s="11"/>
+      <c r="B3" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="32"/>
-      <c r="D3" s="32"/>
-      <c r="E3" s="32"/>
-      <c r="F3" s="32"/>
-      <c r="G3" s="32"/>
-      <c r="H3" s="32"/>
-      <c r="I3" s="32"/>
-      <c r="J3" s="32"/>
-      <c r="K3" s="33"/>
-      <c r="L3" s="13"/>
+      <c r="C3" s="34"/>
+      <c r="D3" s="34"/>
+      <c r="E3" s="34"/>
+      <c r="F3" s="34"/>
+      <c r="G3" s="34"/>
+      <c r="H3" s="34"/>
+      <c r="I3" s="34"/>
+      <c r="J3" s="34"/>
+      <c r="K3" s="35"/>
+      <c r="L3" s="12"/>
     </row>
     <row r="4" spans="1:12" ht="12.75" customHeight="1">
-      <c r="A4" s="6"/>
-      <c r="B4" s="10"/>
-      <c r="C4" s="27"/>
-      <c r="D4" s="27"/>
-      <c r="E4" s="27"/>
-      <c r="F4" s="27"/>
-      <c r="G4" s="27"/>
-      <c r="H4" s="27"/>
-      <c r="I4" s="27"/>
-      <c r="J4" s="10"/>
-      <c r="K4" s="10"/>
-      <c r="L4" s="13"/>
+      <c r="A4" s="5"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="30"/>
+      <c r="F4" s="30"/>
+      <c r="G4" s="30"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="30"/>
+      <c r="J4" s="9"/>
+      <c r="K4" s="9"/>
+      <c r="L4" s="12"/>
     </row>
     <row r="5" spans="1:12" ht="17.45" customHeight="1">
-      <c r="A5" s="6"/>
-      <c r="B5" s="10"/>
-      <c r="C5" s="14" t="s">
+      <c r="A5" s="5"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="14" t="s">
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="H5" s="16"/>
-      <c r="I5" s="10"/>
-      <c r="J5" s="10"/>
-      <c r="K5" s="10"/>
-      <c r="L5" s="13"/>
+      <c r="H5" s="15"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="12"/>
     </row>
     <row r="6" spans="1:12" ht="17.45" customHeight="1">
-      <c r="A6" s="6"/>
-      <c r="B6" s="10"/>
-      <c r="C6" s="14" t="s">
+      <c r="A6" s="5"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="14" t="s">
+      <c r="D6" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="E6" s="10"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="14" t="s">
+      <c r="E6" s="9"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="H6" s="17" t="s">
+      <c r="H6" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="I6" s="10"/>
-      <c r="J6" s="10"/>
-      <c r="K6" s="10"/>
-      <c r="L6" s="13"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="9"/>
+      <c r="K6" s="9"/>
+      <c r="L6" s="12"/>
     </row>
     <row r="7" spans="1:12" ht="12.75" customHeight="1">
-      <c r="A7" s="6"/>
-      <c r="B7" s="10"/>
-      <c r="C7" s="34"/>
-      <c r="D7" s="34"/>
-      <c r="E7" s="34"/>
-      <c r="F7" s="34"/>
-      <c r="G7" s="34"/>
-      <c r="H7" s="10"/>
-      <c r="I7" s="35"/>
-      <c r="J7" s="10"/>
-      <c r="K7" s="10"/>
-      <c r="L7" s="13"/>
+      <c r="A7" s="5"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="28"/>
+      <c r="D7" s="28"/>
+      <c r="E7" s="28"/>
+      <c r="F7" s="28"/>
+      <c r="G7" s="28"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="29"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
+      <c r="L7" s="12"/>
     </row>
     <row r="8" spans="1:12" ht="27.75" customHeight="1">
-      <c r="A8" s="6"/>
+      <c r="A8" s="5"/>
       <c r="B8" s="36" t="s">
         <v>8</v>
       </c>
@@ -2043,10 +2043,10 @@
       <c r="I8" s="37"/>
       <c r="J8" s="37"/>
       <c r="K8" s="38"/>
-      <c r="L8" s="13"/>
+      <c r="L8" s="12"/>
     </row>
     <row r="9" spans="1:12" ht="32.25" customHeight="1">
-      <c r="A9" s="6"/>
+      <c r="A9" s="5"/>
       <c r="B9" s="39" t="s">
         <v>9</v>
       </c>
@@ -2059,83 +2059,83 @@
       <c r="I9" s="40"/>
       <c r="J9" s="40"/>
       <c r="K9" s="41"/>
-      <c r="L9" s="13"/>
+      <c r="L9" s="12"/>
     </row>
     <row r="10" spans="1:12" ht="12.75" customHeight="1">
-      <c r="A10" s="6"/>
-      <c r="B10" s="10"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
-      <c r="E10" s="20"/>
-      <c r="F10" s="20"/>
-      <c r="G10" s="20"/>
-      <c r="H10" s="20"/>
-      <c r="I10" s="20"/>
-      <c r="J10" s="18"/>
-      <c r="K10" s="18"/>
-      <c r="L10" s="13"/>
+      <c r="A10" s="5"/>
+      <c r="B10" s="9"/>
+      <c r="C10" s="19"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="19"/>
+      <c r="F10" s="19"/>
+      <c r="G10" s="19"/>
+      <c r="H10" s="19"/>
+      <c r="I10" s="19"/>
+      <c r="J10" s="17"/>
+      <c r="K10" s="17"/>
+      <c r="L10" s="12"/>
     </row>
     <row r="11" spans="1:12" ht="15.6" customHeight="1">
-      <c r="A11" s="19"/>
-      <c r="B11" s="21" t="s">
+      <c r="A11" s="18"/>
+      <c r="B11" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="21" t="s">
+      <c r="C11" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="D11" s="21" t="s">
+      <c r="D11" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="E11" s="21" t="s">
+      <c r="E11" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="F11" s="21" t="s">
+      <c r="F11" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="G11" s="21" t="s">
+      <c r="G11" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="H11" s="21" t="s">
+      <c r="H11" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="I11" s="21" t="s">
+      <c r="I11" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="J11" s="21" t="s">
+      <c r="J11" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="K11" s="21" t="s">
+      <c r="K11" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="L11" s="22"/>
+      <c r="L11" s="21"/>
     </row>
     <row r="12" spans="1:12" ht="15" customHeight="1">
-      <c r="A12" s="19"/>
-      <c r="B12" s="23"/>
-      <c r="C12" s="23"/>
-      <c r="D12" s="23"/>
-      <c r="E12" s="23"/>
-      <c r="F12" s="23"/>
-      <c r="G12" s="23"/>
-      <c r="H12" s="23"/>
-      <c r="I12" s="23"/>
-      <c r="J12" s="23"/>
-      <c r="K12" s="23"/>
-      <c r="L12" s="22"/>
+      <c r="A12" s="18"/>
+      <c r="B12" s="22"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
+      <c r="G12" s="22"/>
+      <c r="H12" s="22"/>
+      <c r="I12" s="22"/>
+      <c r="J12" s="22"/>
+      <c r="K12" s="22"/>
+      <c r="L12" s="21"/>
     </row>
     <row r="13" spans="1:12" ht="15" customHeight="1">
-      <c r="A13" s="24"/>
-      <c r="B13" s="31"/>
-      <c r="C13" s="25"/>
-      <c r="D13" s="25"/>
-      <c r="E13" s="25"/>
-      <c r="F13" s="25"/>
-      <c r="G13" s="25"/>
-      <c r="H13" s="25"/>
-      <c r="I13" s="25"/>
-      <c r="J13" s="25"/>
-      <c r="K13" s="25"/>
-      <c r="L13" s="26"/>
+      <c r="A13" s="23"/>
+      <c r="B13" s="27"/>
+      <c r="C13" s="24"/>
+      <c r="D13" s="24"/>
+      <c r="E13" s="24"/>
+      <c r="F13" s="24"/>
+      <c r="G13" s="24"/>
+      <c r="H13" s="24"/>
+      <c r="I13" s="24"/>
+      <c r="J13" s="24"/>
+      <c r="K13" s="24"/>
+      <c r="L13" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>